<commit_message>
Minor change dpe ERC mortality
no impact on harmonized dataset
</commit_message>
<xml_diff>
--- a/mortality/data_processing_elements_mortality-ERC.xlsx
+++ b/mortality/data_processing_elements_mortality-ERC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Melchias\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Melchias\Downloads\harmonization_linkage_ERC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3E558F-6FBD-4E00-A7D8-A8FED24AECA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0200E2-A4C9-4B77-8920-34022500EDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="885" yWindow="690" windowWidth="26370" windowHeight="16695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="2355" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="78">
   <si>
     <t>index</t>
   </si>
@@ -241,9 +241,6 @@
   </si>
   <si>
     <t>dataschema_variable</t>
-  </si>
-  <si>
-    <t>bcsid</t>
   </si>
   <si>
     <t>"ERC"</t>
@@ -857,7 +854,7 @@
         <v>24</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="O2" s="7"/>
       <c r="R2" s="7" t="s">
@@ -870,7 +867,7 @@
         <v>27</v>
       </c>
       <c r="U2" s="7" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.25">
@@ -909,7 +906,7 @@
         <v>33</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:58" x14ac:dyDescent="0.25">
@@ -948,7 +945,7 @@
         <v>33</v>
       </c>
       <c r="U4" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:58" x14ac:dyDescent="0.25">
@@ -984,7 +981,7 @@
         <v>33</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:58" x14ac:dyDescent="0.25">
@@ -1097,13 +1094,13 @@
         <v>42</v>
       </c>
       <c r="M8" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="O8" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="N8" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="O8" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="P8" s="7" t="s">
         <v>48</v>
@@ -1118,7 +1115,7 @@
         <v>41</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="V8" s="9"/>
       <c r="W8" s="9"/>
@@ -1323,7 +1320,7 @@
         <v>38</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="O11" s="7"/>
       <c r="R11" s="7" t="s">
@@ -1333,10 +1330,10 @@
         <v>40</v>
       </c>
       <c r="T11" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="V11" s="9"/>
       <c r="W11" s="9"/>

</xml_diff>